<commit_message>
Rebuild all 9 templates to professional quality - formulas, instructions tabs, trade-specific data, proper formatting
</commit_message>
<xml_diff>
--- a/downloads/change-order.xlsx
+++ b/downloads/change-order.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Order" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Order" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,9 +32,10 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00F97316"/>
-      <sz val="24"/>
-    </font>
-    <font>
+      <sz val="28"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="14"/>
     </font>
@@ -44,6 +46,29 @@
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <color rgb="00333333"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00F97316"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00F97316"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00F97316"/>
       <sz val="12"/>
@@ -51,24 +76,22 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
+      <color rgb="00F97316"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00F97316"/>
-      <sz val="13"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -87,6 +110,12 @@
         <bgColor rgb="00F8FAFC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF7ED"/>
+        <bgColor rgb="00FFF7ED"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -97,39 +126,56 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color rgb="00D1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -492,299 +538,327 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00F97316"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>📋 Change Order Template — Instructions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>BuiltRight Academy | builtrighthq.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>— Always document scope changes in writing before doing the work. —</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>© 2026 BuiltRight Academy | builtrighthq.com</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00F97316"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>CHANGE ORDER</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>YOUR COMPANY NAME</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Change Order #:</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>[YOUR COMPANY NAME]</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>CO #:</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>CO-001</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>(555) 123-4567 | info@yourcompany.com</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>Date:</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>03/09/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Original Contract #:</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>PROP-2026-015</t>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Original Contract:</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>PROP-2026-018</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>CLIENT:</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Client Name</t>
-        </is>
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Original Amount:</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>10315</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>PROJECT:</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Basement Finishing</t>
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Client:</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Robert &amp; Maria Garcia</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>ORIGINAL CONTRACT AMOUNT:</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>31350</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>DESCRIPTION OF CHANGES</t>
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>REASON FOR CHANGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="50" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>During demo, discovered water damage behind shower wall requiring additional repair before tile installation. Client also requested upgrade from standard to heated tile floor.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Client requests the following additions/modifications to the original scope:</t>
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>CHANGES</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Hours/Qty</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Amount</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>Item Added / Removed</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>Replace rotted studs (3) and subfloor section</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>Add</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>Deduct</t>
-        </is>
+      <c r="C15" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="14" t="n">
+        <v>450</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="n">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>Mold remediation — treat &amp; seal affected area</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>Add wet bar with sink in living area</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="n">
-        <v>3200</v>
-      </c>
-      <c r="D16" s="9" t="inlineStr"/>
+      <c r="D16" s="17" t="n">
+        <v>350</v>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>Upgrade flooring from LVP to engineered hardwood</t>
-        </is>
-      </c>
-      <c r="C17" s="12" t="n">
-        <v>1800</v>
-      </c>
-      <c r="D17" s="12" t="inlineStr"/>
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>Heated floor mat — Nuheat 35 sq ft + thermostat</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="14" t="n">
+        <v>680</v>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Add egress window to bedroom 2</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="n">
-        <v>2400</v>
-      </c>
-      <c r="D18" s="9" t="inlineStr"/>
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>Heated floor installation labor</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" s="17" t="n">
+        <v>280</v>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>Remove built-in shelving from original scope</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="inlineStr"/>
-      <c r="D19" s="12" t="n">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>Add recessed lighting (4 additional cans)</t>
-        </is>
-      </c>
-      <c r="C20" s="9" t="n">
-        <v>680</v>
-      </c>
-      <c r="D20" s="9" t="inlineStr"/>
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>Standard tile installation labor (reduced — partial overlap)</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>Remove</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="14" t="n">
+        <v>-120</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Net Change:</t>
+        </is>
+      </c>
+      <c r="D21" s="18">
+        <f>SUM(D15:D20)</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Total Additions:</t>
-        </is>
-      </c>
-      <c r="C22" s="4">
-        <f>SUM(C16:C20)</f>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>New Total:</t>
+        </is>
+      </c>
+      <c r="D22" s="19">
+        <f>B7+D21</f>
         <v/>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Total Deductions:</t>
-        </is>
-      </c>
-      <c r="D23" s="4">
-        <f>SUM(D16:D20)</f>
-        <v/>
-      </c>
-    </row>
     <row r="24">
-      <c r="B24" s="13" t="inlineStr">
-        <is>
-          <t>Net Change:</t>
-        </is>
-      </c>
-      <c r="C24" s="14">
-        <f>C22-D23</f>
-        <v/>
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Timeline Impact: Adds approximately 2 additional work days.</t>
+        </is>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="15" t="inlineStr">
-        <is>
-          <t>NEW CONTRACT TOTAL:</t>
-        </is>
-      </c>
-      <c r="C26" s="16">
-        <f>C10+C24</f>
-        <v/>
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>AUTHORIZATION</t>
+        </is>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>Schedule Impact:</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Add 5 working days</t>
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Client Signature: _______________________  Date: ____________</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>APPROVAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Both parties agree to the changes described above.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Client Signature: ____________________________    Date: ____________</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Contractor Signature: ________________________    Date: ____________</t>
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Contractor Signature: ____________________  Date: ____________</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A13:D13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>